<commit_message>
BOM and PCB edited for Nano every
</commit_message>
<xml_diff>
--- a/system_design/Georgetown/V0.5.2/bill_of_materials.xlsx
+++ b/system_design/Georgetown/V0.5.2/bill_of_materials.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://emailsc-my.sharepoint.com/personal/asifuzzaman_sc_edu/Documents/Github Repos/UAV-Deployable-Stage-Height-Sensor/system_design/Georgetown/V0.5.2/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="10" documentId="13_ncr:1_{D03FB38C-2BB2-4F7F-8258-5EC3F0FCDEF0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A280CD80-4589-40BA-AB22-9C2530583FA7}"/>
+  <xr:revisionPtr revIDLastSave="19" documentId="13_ncr:1_{D03FB38C-2BB2-4F7F-8258-5EC3F0FCDEF0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{361C4FFD-C589-477A-8659-487DD38F222F}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-16320" windowWidth="29040" windowHeight="15720" xr2:uid="{FDAE7DA4-9528-4FC7-A320-70DA50473DCE}"/>
   </bookViews>
@@ -36,10 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="190" uniqueCount="153">
-  <si>
-    <t>Arduino Nano</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="189" uniqueCount="153">
   <si>
     <t>NRF24L01+ 2.4GHz Wireless RF Transceiver Module</t>
   </si>
@@ -92,9 +89,6 @@
     <t>Individual Cost</t>
   </si>
   <si>
-    <t>https://store-usa.arduino.cc/products/arduino-nano?utm_source=google&amp;utm_medium=cpc&amp;utm_campaign=US-Pmax&amp;gad_source=1&amp;gclid=CjwKCAjw7pO_BhAlEiwA4pMQvGgjSAL_aiPDuQtjDtxsbhZPY6NtgwMyrIq1obT8kDad0uOfvd-_6xoCrvUQAvD_BwE</t>
-  </si>
-  <si>
     <t>https://www.amazon.com/Makerfire-Arduino-NRF24L01-Wireless-Transceiver/dp/B00O9O868G/ref=asc_df_B00O9O868G?mcid=dab308f0de3430dfa5c9f8399ca22b35&amp;hvocijid=9184541888213339040-B00O9O868G-&amp;hvexpln=73&amp;tag=hyprod-20&amp;linkCode=df0&amp;hvadid=721245378154&amp;hvpos=&amp;hvnetw=g&amp;hvrand=9184541888213339040&amp;hvpone=&amp;hvptwo=&amp;hvqmt=&amp;hvdev=c&amp;hvdvcmdl=&amp;hvlocint=&amp;hvlocphy=9198699&amp;hvtargid=pla-2281435177578&amp;psc=1</t>
   </si>
   <si>
@@ -197,12 +191,6 @@
     <t>Vendor 3</t>
   </si>
   <si>
-    <t>https://www.digikey.com/en/products/detail/arduino/A000005/2638989?gclsrc=aw.ds&amp;gad_source=1&amp;gad_campaignid=20243136172&amp;gbraid=0AAAAADrbLli4_Ap0H678W2amsXvkFFD8z&amp;gclid=EAIaIQobChMI7K31g6HsjQMVtUP_AR30cCLzEAQYBCABEgJLw_D_BwE</t>
-  </si>
-  <si>
-    <t>https://www.ebay.com/itm/254630577493?chn=ps&amp;mkevt=1&amp;mkcid=28&amp;google_free_listing_action=view_item&amp;srsltid=AfmBOorV61PA8LrmcVCLmkRxgli-ic749EmEj9uG3olJqtVqK8C26RwUy3g&amp;gQT=2</t>
-  </si>
-  <si>
     <t>https://www.ebay.com/itm/235081679206?chn=ps&amp;var=536091370095&amp;norover=1&amp;mkevt=1&amp;mkrid=711-117182-37290-0&amp;mkcid=2&amp;mkscid=101&amp;itemid=536091370095_235081679206&amp;targetid=2295557532710&amp;device=c&amp;mktype=pla&amp;googleloc=9198699&amp;poi=&amp;campaignid=21400677539&amp;mkgroupid=173029508628&amp;rlsatarget=pla-2295557532710&amp;abcId=9448483&amp;merchantid=734150552&amp;gad_source=1&amp;gad_campaignid=21400677539&amp;gbraid=0AAAAAD_QDh9KZSet77KcrE8f9gL7cL_CG&amp;gclid=EAIaIQobChMIi8KGzaPsjQMVGEf_AR2yNzdrEAQYAyABEgL6F_D_BwE</t>
   </si>
   <si>
@@ -495,6 +483,18 @@
   </si>
   <si>
     <t xml:space="preserve"> BME280 Pressure, Temperature and Humidity sensor</t>
+  </si>
+  <si>
+    <t>Arduino Nano every</t>
+  </si>
+  <si>
+    <t>https://store-usa.arduino.cc/products/nano-every?srsltid=AU7gw4VAi4WgP3ovYMnTBXjmXlqWVpI_EFwJ743bYmzsuLMy5s4qXwGh</t>
+  </si>
+  <si>
+    <t>https://www.sparkfun.com/arduino-nano-every.html?utm_source=google&amp;utm_medium=cpc&amp;utm_campaign=Generic+%7C+PMax&amp;utm_content=Full+Catalog&amp;gad_source=1&amp;gad_campaignid=17479024039&amp;gbraid=0AAAAADsj4ET0NZro45iUWdM-Ba6AQ0YWk&amp;gclid=CjwKCAjw_KjVBhAHEiwAnC0N9MHYi96OUVs8ZOLr9cRyVdCITPEBJ4SesPMJTw66NdfeWCyuEPozBxoCvzYQAvD_BwE</t>
+  </si>
+  <si>
+    <t>Nano every</t>
   </si>
 </sst>
 </file>
@@ -942,87 +942,85 @@
   <sheetData>
     <row r="1" spans="1:13" s="6" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="5" t="s">
-        <v>148</v>
+        <v>144</v>
       </c>
       <c r="B1" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="C1" s="5" t="s">
+        <v>145</v>
+      </c>
+      <c r="D1" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="C1" s="5" t="s">
-        <v>149</v>
-      </c>
-      <c r="D1" s="5" t="s">
+      <c r="E1" s="5" t="s">
+        <v>117</v>
+      </c>
+      <c r="F1" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="E1" s="5" t="s">
-        <v>121</v>
-      </c>
-      <c r="F1" s="5" t="s">
-        <v>17</v>
-      </c>
       <c r="G1" s="5" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="H1" s="5" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="I1" s="5" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="J1" s="5" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="K1" s="5" t="s">
-        <v>85</v>
+        <v>81</v>
       </c>
       <c r="L1" s="5" t="s">
-        <v>86</v>
+        <v>82</v>
       </c>
       <c r="M1" s="5" t="s">
-        <v>87</v>
+        <v>83</v>
       </c>
     </row>
     <row r="2" spans="1:13" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" s="2" t="s">
-        <v>0</v>
+        <v>152</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>0</v>
+        <v>149</v>
       </c>
       <c r="D2" s="2">
         <v>1</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
       <c r="F2" s="3">
-        <v>25.7</v>
+        <v>12.9</v>
       </c>
       <c r="G2" s="3">
         <f>D2*F2</f>
-        <v>25.7</v>
+        <v>12.9</v>
       </c>
       <c r="H2" s="1" t="s">
-        <v>18</v>
+        <v>150</v>
       </c>
       <c r="I2" s="1" t="s">
-        <v>53</v>
-      </c>
-      <c r="J2" s="1" t="s">
-        <v>54</v>
-      </c>
+        <v>151</v>
+      </c>
+      <c r="J2" s="1"/>
     </row>
     <row r="3" spans="1:13" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
-        <v>119</v>
+        <v>115</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>105</v>
+        <v>101</v>
       </c>
       <c r="D3" s="2">
         <v>1</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
       <c r="F3" s="3">
         <v>2.52</v>
@@ -1032,24 +1030,24 @@
         <v>2.52</v>
       </c>
       <c r="H3" s="1" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="I3" s="1" t="s">
-        <v>55</v>
+        <v>51</v>
       </c>
     </row>
     <row r="4" spans="1:13" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A4" s="2" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D4" s="2">
         <v>1</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
       <c r="F4" s="3">
         <v>1.4</v>
@@ -1059,27 +1057,27 @@
         <v>1.4</v>
       </c>
       <c r="H4" s="1" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="I4" s="1" t="s">
-        <v>56</v>
+        <v>52</v>
       </c>
       <c r="J4" s="2" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
     </row>
     <row r="5" spans="1:13" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A5" s="2" t="s">
-        <v>118</v>
+        <v>114</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>106</v>
+        <v>102</v>
       </c>
       <c r="D5" s="2">
         <v>1</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
       <c r="F5" s="3">
         <v>11.96</v>
@@ -1089,24 +1087,24 @@
         <v>11.96</v>
       </c>
       <c r="H5" s="1" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="I5" s="1" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
     </row>
     <row r="6" spans="1:13" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A6" s="2" t="s">
-        <v>107</v>
+        <v>103</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>152</v>
+        <v>148</v>
       </c>
       <c r="D6" s="2">
         <v>1</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
       <c r="F6" s="3">
         <v>5.26</v>
@@ -1116,33 +1114,33 @@
         <v>5.26</v>
       </c>
       <c r="H6" s="1" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="I6" s="1" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="J6" s="1" t="s">
-        <v>59</v>
+        <v>55</v>
       </c>
       <c r="K6" s="1" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="L6" s="1" t="s">
-        <v>147</v>
+        <v>143</v>
       </c>
     </row>
     <row r="7" spans="1:13" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A7" s="2" t="s">
-        <v>145</v>
+        <v>141</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>131</v>
+        <v>127</v>
       </c>
       <c r="D7" s="2">
         <v>1</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
       <c r="F7" s="3">
         <v>4.95</v>
@@ -1152,24 +1150,24 @@
         <v>4.95</v>
       </c>
       <c r="H7" s="1" t="s">
-        <v>132</v>
+        <v>128</v>
       </c>
       <c r="I7" s="1" t="s">
-        <v>133</v>
+        <v>129</v>
       </c>
     </row>
     <row r="8" spans="1:13" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A8" s="2" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D8" s="2">
         <v>1</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
       <c r="F8" s="3">
         <v>15.2</v>
@@ -1179,21 +1177,21 @@
         <v>15.2</v>
       </c>
       <c r="H8" s="1" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
     </row>
     <row r="9" spans="1:13" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A9" s="2" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="D9" s="2">
         <v>1</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
       <c r="F9" s="3">
         <v>5.25</v>
@@ -1203,27 +1201,27 @@
         <v>5.25</v>
       </c>
       <c r="H9" s="1" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="I9" s="2" t="s">
-        <v>61</v>
+        <v>57</v>
       </c>
       <c r="J9" s="2" t="s">
-        <v>62</v>
+        <v>58</v>
       </c>
     </row>
     <row r="10" spans="1:13" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A10" s="2" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>90</v>
+        <v>86</v>
       </c>
       <c r="D10" s="2">
         <v>1</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
       <c r="F10" s="3">
         <v>18</v>
@@ -1233,25 +1231,25 @@
         <v>18</v>
       </c>
       <c r="H10" s="1" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="I10" s="1" t="s">
-        <v>150</v>
+        <v>146</v>
       </c>
       <c r="J10" s="1"/>
     </row>
     <row r="11" spans="1:13" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A11" s="2" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D11" s="2">
         <v>1</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
       <c r="F11" s="3">
         <v>1.0900000000000001</v>
@@ -1261,24 +1259,24 @@
         <v>1.0900000000000001</v>
       </c>
       <c r="H11" s="1" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="I11" s="2" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
     </row>
     <row r="12" spans="1:13" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A12" s="2" t="s">
-        <v>108</v>
+        <v>104</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D12" s="2">
         <v>1</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
       <c r="F12" s="3">
         <v>0.57999999999999996</v>
@@ -1288,24 +1286,24 @@
         <v>0.57999999999999996</v>
       </c>
       <c r="H12" s="1" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="I12" s="2" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
     </row>
     <row r="13" spans="1:13" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A13" s="2" t="s">
-        <v>141</v>
+        <v>137</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>144</v>
+        <v>140</v>
       </c>
       <c r="D13" s="2">
         <v>1</v>
       </c>
       <c r="E13" s="2" t="s">
-        <v>142</v>
+        <v>138</v>
       </c>
       <c r="F13" s="3">
         <v>0.14000000000000001</v>
@@ -1315,21 +1313,21 @@
         <v>0.14000000000000001</v>
       </c>
       <c r="H13" s="1" t="s">
-        <v>143</v>
+        <v>139</v>
       </c>
     </row>
     <row r="14" spans="1:13" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A14" s="2" t="s">
-        <v>146</v>
+        <v>142</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D14" s="2">
         <v>1</v>
       </c>
       <c r="E14" s="2" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
       <c r="F14" s="3">
         <v>8.23</v>
@@ -1339,21 +1337,21 @@
         <v>8.23</v>
       </c>
       <c r="H14" s="1" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
     </row>
     <row r="15" spans="1:13" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A15" s="2" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>114</v>
+        <v>110</v>
       </c>
       <c r="D15" s="2">
         <v>1</v>
       </c>
       <c r="E15" s="2" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
       <c r="F15" s="3">
         <v>8.24</v>
@@ -1363,36 +1361,36 @@
         <v>8.24</v>
       </c>
       <c r="H15" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="I15" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="J15" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="K15" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="L15" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="M15" s="2" t="s">
         <v>80</v>
-      </c>
-      <c r="I15" s="1" t="s">
-        <v>81</v>
-      </c>
-      <c r="J15" s="1" t="s">
-        <v>82</v>
-      </c>
-      <c r="K15" s="1" t="s">
-        <v>83</v>
-      </c>
-      <c r="L15" s="2" t="s">
-        <v>65</v>
-      </c>
-      <c r="M15" s="2" t="s">
-        <v>84</v>
       </c>
     </row>
     <row r="16" spans="1:13" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A16" s="2" t="s">
-        <v>109</v>
+        <v>105</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>110</v>
+        <v>106</v>
       </c>
       <c r="D16" s="2">
         <v>1</v>
       </c>
       <c r="E16" s="2" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
       <c r="F16" s="3">
         <v>2.0299999999999998</v>
@@ -1402,24 +1400,24 @@
         <v>2.0299999999999998</v>
       </c>
       <c r="H16" s="1" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="I16" s="2" t="s">
-        <v>66</v>
+        <v>62</v>
       </c>
     </row>
     <row r="17" spans="1:10" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A17" s="2" t="s">
-        <v>115</v>
+        <v>111</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>99</v>
+        <v>95</v>
       </c>
       <c r="D17" s="2">
         <v>1</v>
       </c>
       <c r="E17" s="2" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
       <c r="F17" s="3">
         <v>0.2</v>
@@ -1429,24 +1427,24 @@
         <v>0.2</v>
       </c>
       <c r="H17" s="1" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="I17" s="2" t="s">
-        <v>67</v>
+        <v>63</v>
       </c>
     </row>
     <row r="18" spans="1:10" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A18" s="2" t="s">
-        <v>137</v>
+        <v>133</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>138</v>
+        <v>134</v>
       </c>
       <c r="D18" s="2">
         <v>3</v>
       </c>
       <c r="E18" s="2" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
       <c r="F18" s="3">
         <v>0.1</v>
@@ -1456,21 +1454,21 @@
         <v>0.30000000000000004</v>
       </c>
       <c r="H18" s="1" t="s">
-        <v>139</v>
+        <v>135</v>
       </c>
     </row>
     <row r="19" spans="1:10" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A19" s="2" t="s">
-        <v>100</v>
+        <v>96</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="D19" s="2">
         <v>3</v>
       </c>
       <c r="E19" s="2" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
       <c r="F19" s="3">
         <v>0.1</v>
@@ -1480,24 +1478,24 @@
         <v>0.30000000000000004</v>
       </c>
       <c r="H19" s="1" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="I19" s="1" t="s">
-        <v>68</v>
+        <v>64</v>
       </c>
     </row>
     <row r="20" spans="1:10" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A20" s="2" t="s">
-        <v>101</v>
+        <v>97</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="D20" s="2">
         <v>4</v>
       </c>
       <c r="E20" s="2" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
       <c r="F20" s="3">
         <v>0.1</v>
@@ -1507,24 +1505,24 @@
         <v>0.4</v>
       </c>
       <c r="H20" s="1" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="I20" s="2" t="s">
-        <v>69</v>
+        <v>65</v>
       </c>
     </row>
     <row r="21" spans="1:10" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A21" s="2" t="s">
-        <v>134</v>
+        <v>130</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
       <c r="D21" s="2">
         <v>2</v>
       </c>
       <c r="E21" s="2" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
       <c r="F21" s="3">
         <v>0.1</v>
@@ -1534,21 +1532,21 @@
         <v>0.2</v>
       </c>
       <c r="H21" s="1" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
     </row>
     <row r="22" spans="1:10" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A22" s="2" t="s">
-        <v>102</v>
+        <v>98</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>94</v>
+        <v>90</v>
       </c>
       <c r="D22" s="2">
         <v>1</v>
       </c>
       <c r="E22" s="2" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
       <c r="F22" s="3">
         <v>0.39</v>
@@ -1558,24 +1556,24 @@
         <v>0.39</v>
       </c>
       <c r="H22" s="1" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="I22" s="2" t="s">
-        <v>70</v>
+        <v>66</v>
       </c>
     </row>
     <row r="23" spans="1:10" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A23" s="2" t="s">
-        <v>103</v>
+        <v>99</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>95</v>
+        <v>91</v>
       </c>
       <c r="D23" s="2">
         <v>1</v>
       </c>
       <c r="E23" s="2" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
       <c r="F23" s="3">
         <v>0.41</v>
@@ -1585,24 +1583,24 @@
         <v>0.41</v>
       </c>
       <c r="H23" s="1" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="I23" s="2" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
     </row>
     <row r="24" spans="1:10" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A24" s="2" t="s">
-        <v>98</v>
+        <v>94</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
       <c r="D24" s="2">
         <v>1</v>
       </c>
       <c r="E24" s="2" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
       <c r="F24" s="3">
         <v>0.26</v>
@@ -1612,24 +1610,24 @@
         <v>0.26</v>
       </c>
       <c r="H24" s="1" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="I24" s="2" t="s">
-        <v>72</v>
+        <v>68</v>
       </c>
     </row>
     <row r="25" spans="1:10" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A25" s="2" t="s">
-        <v>140</v>
+        <v>136</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="D25" s="2">
         <v>4</v>
       </c>
       <c r="E25" s="2" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
       <c r="F25" s="3">
         <v>0.48</v>
@@ -1639,24 +1637,24 @@
         <v>1.92</v>
       </c>
       <c r="H25" s="1" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="I25" s="2" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
     </row>
     <row r="26" spans="1:10" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A26" s="2" t="s">
-        <v>104</v>
+        <v>100</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>97</v>
+        <v>93</v>
       </c>
       <c r="D26" s="2">
         <v>1</v>
       </c>
       <c r="E26" s="2" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
       <c r="F26" s="3">
         <v>3.58</v>
@@ -1666,27 +1664,27 @@
         <v>3.58</v>
       </c>
       <c r="H26" s="1" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="I26" s="1" t="s">
-        <v>74</v>
+        <v>70</v>
       </c>
       <c r="J26" s="2" t="s">
-        <v>75</v>
+        <v>71</v>
       </c>
     </row>
     <row r="27" spans="1:10" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A27" s="2" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D27" s="2">
         <v>1</v>
       </c>
       <c r="E27" s="2" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
       <c r="F27" s="3">
         <v>60.76</v>
@@ -1696,21 +1694,21 @@
         <v>60.76</v>
       </c>
       <c r="H27" s="1" t="s">
-        <v>76</v>
+        <v>72</v>
       </c>
     </row>
     <row r="28" spans="1:10" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A28" s="2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>113</v>
+        <v>109</v>
       </c>
       <c r="D28" s="2">
         <v>1</v>
       </c>
       <c r="E28" s="2" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
       <c r="F28" s="3">
         <v>0.91</v>
@@ -1720,24 +1718,24 @@
         <v>0.91</v>
       </c>
       <c r="H28" s="1" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="I28" s="2" t="s">
-        <v>77</v>
+        <v>73</v>
       </c>
     </row>
     <row r="29" spans="1:10" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A29" s="2" t="s">
-        <v>111</v>
+        <v>107</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="D29" s="2">
         <v>1</v>
       </c>
       <c r="E29" s="2" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
       <c r="F29" s="3">
         <v>2.15</v>
@@ -1747,24 +1745,24 @@
         <v>2.15</v>
       </c>
       <c r="H29" s="1" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="I29" s="2" t="s">
-        <v>78</v>
+        <v>74</v>
       </c>
     </row>
     <row r="30" spans="1:10" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A30" s="2" t="s">
-        <v>127</v>
+        <v>123</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>129</v>
+        <v>125</v>
       </c>
       <c r="D30" s="2">
         <v>1</v>
       </c>
       <c r="E30" s="2" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
       <c r="F30" s="3">
         <v>0.1</v>
@@ -1774,21 +1772,21 @@
         <v>0.1</v>
       </c>
       <c r="H30" s="1" t="s">
-        <v>128</v>
+        <v>124</v>
       </c>
     </row>
     <row r="31" spans="1:10" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A31" s="2" t="s">
-        <v>130</v>
+        <v>126</v>
       </c>
       <c r="B31" s="2" t="s">
-        <v>112</v>
+        <v>108</v>
       </c>
       <c r="D31" s="2">
         <v>1</v>
       </c>
       <c r="E31" s="2" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
       <c r="F31" s="3">
         <v>0.13</v>
@@ -1798,24 +1796,24 @@
         <v>0.13</v>
       </c>
       <c r="H31" s="1" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="I31" s="2" t="s">
-        <v>79</v>
+        <v>75</v>
       </c>
     </row>
     <row r="32" spans="1:10" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A32" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="B32" s="2" t="s">
         <v>39</v>
-      </c>
-      <c r="B32" s="2" t="s">
-        <v>41</v>
       </c>
       <c r="D32" s="2">
         <v>9</v>
       </c>
       <c r="E32" s="2" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
       <c r="F32" s="3">
         <v>7.39</v>
@@ -1825,18 +1823,18 @@
         <v>66.509999999999991</v>
       </c>
       <c r="H32" s="1" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
     </row>
     <row r="33" spans="1:8" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B33" s="2" t="s">
-        <v>125</v>
+        <v>121</v>
       </c>
       <c r="D33" s="2">
         <v>2</v>
       </c>
       <c r="E33" s="2" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
       <c r="F33" s="3">
         <v>0.01</v>
@@ -1849,13 +1847,13 @@
     </row>
     <row r="34" spans="1:8" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B34" s="2" t="s">
-        <v>126</v>
+        <v>122</v>
       </c>
       <c r="D34" s="2">
         <v>2</v>
       </c>
       <c r="E34" s="2" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
       <c r="F34" s="3">
         <v>0.01</v>
@@ -1868,13 +1866,13 @@
     </row>
     <row r="35" spans="1:8" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B35" s="2" t="s">
-        <v>123</v>
+        <v>119</v>
       </c>
       <c r="D35" s="2">
         <v>2</v>
       </c>
       <c r="E35" s="2" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
       <c r="F35" s="3">
         <v>0.01</v>
@@ -1884,18 +1882,18 @@
         <v>0.02</v>
       </c>
       <c r="H35" s="1" t="s">
-        <v>120</v>
+        <v>116</v>
       </c>
     </row>
     <row r="36" spans="1:8" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B36" s="2" t="s">
-        <v>124</v>
+        <v>120</v>
       </c>
       <c r="D36" s="2">
         <v>4</v>
       </c>
       <c r="E36" s="2" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
       <c r="F36" s="3">
         <v>7.2999999999999995E-2</v>
@@ -1905,21 +1903,21 @@
         <v>0.29199999999999998</v>
       </c>
       <c r="H36" s="1" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
     </row>
     <row r="37" spans="1:8" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A37" s="2" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="B37" s="2" t="s">
-        <v>116</v>
+        <v>112</v>
       </c>
       <c r="D37" s="2">
         <v>1</v>
       </c>
       <c r="E37" s="2" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
       <c r="F37" s="3">
         <v>2.68</v>
@@ -1929,21 +1927,21 @@
         <v>2.68</v>
       </c>
       <c r="H37" s="1" t="s">
-        <v>117</v>
+        <v>113</v>
       </c>
     </row>
     <row r="38" spans="1:8" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A38" s="2" t="s">
-        <v>91</v>
+        <v>87</v>
       </c>
       <c r="B38" s="2" t="s">
-        <v>92</v>
+        <v>88</v>
       </c>
       <c r="D38" s="2">
         <v>1</v>
       </c>
       <c r="E38" s="2" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
       <c r="F38" s="3">
         <v>25</v>
@@ -1953,72 +1951,71 @@
         <v>25</v>
       </c>
       <c r="H38" s="1" t="s">
-        <v>93</v>
+        <v>89</v>
       </c>
     </row>
     <row r="39" spans="1:8" x14ac:dyDescent="0.35">
       <c r="F39" s="4" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G39" s="4">
         <f>SUM(G2:G38)</f>
-        <v>277.10200000000003</v>
+        <v>264.30200000000002</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="H2" r:id="rId1" xr:uid="{42481F3C-D77C-4D47-8482-158A61C0337E}"/>
-    <hyperlink ref="H4" r:id="rId2" display="https://www.amazon.com/Makerfire-Arduino-NRF24L01-Wireless-Transceiver/dp/B00O9O868G/ref=asc_df_B00O9O868G?mcid=dab308f0de3430dfa5c9f8399ca22b35&amp;hvocijid=9184541888213339040-B00O9O868G-&amp;hvexpln=73&amp;tag=hyprod-20&amp;linkCode=df0&amp;hvadid=721245378154&amp;hvpos=&amp;hvnetw=g&amp;hvrand=9184541888213339040&amp;hvpone=&amp;hvptwo=&amp;hvqmt=&amp;hvdev=c&amp;hvdvcmdl=&amp;hvlocint=&amp;hvlocphy=9198699&amp;hvtargid=pla-2281435177578&amp;psc=1" xr:uid="{89AEDB65-21E6-41D2-A940-81A81142AD5C}"/>
-    <hyperlink ref="H5" r:id="rId3" xr:uid="{E70F36E4-82C7-490A-965C-FBA0B568208C}"/>
-    <hyperlink ref="I6" r:id="rId4" display="https://www.amazon.com/Onyehn-Temperature-Humidity-Barometric-Pressure/dp/B07KR24P6P/ref=asc_df_B07KR24P6P?mcid=2faf80a473c33e3bb7b53dc75a65a9ac&amp;hvocijid=2199110702432476394-B07KR24P6P-&amp;hvexpln=73&amp;tag=hyprod-20&amp;linkCode=df0&amp;hvadid=721245378154&amp;hvpos=&amp;hvnetw=g&amp;hvrand=2199110702432476394&amp;hvpone=&amp;hvptwo=&amp;hvqmt=&amp;hvdev=c&amp;hvdvcmdl=&amp;hvlocint=&amp;hvlocphy=9198699&amp;hvtargid=pla-2281435177578&amp;psc=1" xr:uid="{04CEC65C-3665-4D25-B259-AF9E667F3BA6}"/>
-    <hyperlink ref="H8" r:id="rId5" xr:uid="{23E423E1-1EBE-4115-AE06-49032C41D232}"/>
-    <hyperlink ref="H9" r:id="rId6" display="https://www.sparkfun.com/ultrasonic-distance-sensor-hc-sr04.html" xr:uid="{F999829F-3DFC-4DBA-B819-1D673798FA55}"/>
-    <hyperlink ref="H10" r:id="rId7" display="https://zeeebattery.com/products/zeee-7-4v-60c-1500mah-2s-lipo-battery-deans-plug?variant=43953770299699&amp;country=US&amp;currency=USD&amp;utm_medium=product_sync&amp;utm_source=google&amp;utm_content=sag_organic&amp;utm_campaign=sag_organic&amp;gad_source=1&amp;gclid=CjwKCAjw7pO_BhAlEiwA4pMQvJInDAYww1F-RyBS_FKHJZs2q-GgKMjZj0IEfHsjSMYCjfxmAI9laxoCeRQQAvD_BwE" xr:uid="{BB8CB9D1-9310-4C54-A510-64D6DA058543}"/>
-    <hyperlink ref="H11" r:id="rId8" display="https://www.digikey.com/en/products/detail/jauch-quartz/CR1025/16399048" xr:uid="{17A29435-522E-4BB5-8364-3BC77FBEB1C4}"/>
-    <hyperlink ref="H12" r:id="rId9" display="https://www.digikey.com/en/products/detail/mpd-memory-protection-devices/bk-870/3829737" xr:uid="{27F9BEB5-8046-41B8-A401-6B801AA65292}"/>
-    <hyperlink ref="H17" r:id="rId10" display="https://www.digikey.com/en/products/detail/american-opto-plus-led/L314ED/13677700?s=N4IgTCBcDaIDIGYCMAWAogERAXQL5A" xr:uid="{EB1FB783-CD78-4F2E-ADAE-2EFC2E0C050D}"/>
-    <hyperlink ref="H20" r:id="rId11" xr:uid="{1CE23A94-3355-4CE3-BD99-944097BF2C76}"/>
-    <hyperlink ref="H25" r:id="rId12" display="https://www.digikey.com/en/products/detail/kemet/c1206s104k5racauto/10232834" xr:uid="{CDDFAE49-11BE-4283-9E44-D17951ACE335}"/>
-    <hyperlink ref="H26" r:id="rId13" display="https://www.digikey.com/en/products/detail/microchip-technology/mic5239-5-0ys-tr/2346595" xr:uid="{0FF0C8FA-B521-42B4-9637-4551CDF56AE0}"/>
-    <hyperlink ref="H28" r:id="rId14" display="https://www.digikey.com/en/products/detail/samtec-inc/ssa-104-w-t/1105908" xr:uid="{5CEFEAD0-E765-4C5C-8B17-4D481AAEE74F}"/>
-    <hyperlink ref="H14" r:id="rId15" xr:uid="{98CBDFFF-5BC0-4691-985C-193C55CD2A4F}"/>
-    <hyperlink ref="H16" r:id="rId16" xr:uid="{F40F3420-CF30-4700-92F3-040B50F37E84}"/>
-    <hyperlink ref="H23" r:id="rId17" xr:uid="{CF84383E-32DC-4F7A-8B1F-D5487EDC174E}"/>
-    <hyperlink ref="H24" r:id="rId18" xr:uid="{9AFC6348-0E57-4A67-A197-41D4FD45794D}"/>
-    <hyperlink ref="H3" r:id="rId19" xr:uid="{132AA37F-9E12-44EF-9546-36BDCE2F9F6B}"/>
-    <hyperlink ref="H32" r:id="rId20" xr:uid="{BECD5DE6-8852-4EA8-869E-7E18A46D5C74}"/>
-    <hyperlink ref="H31" r:id="rId21" display="https://www.digikey.com/en/products/detail/jst-sales-america-inc/B3B-XH-A/1651046?gad_source=1&amp;gad_campaignid=20470400566&amp;gbraid=0AAAAADrbLlgCz6Py2S0va5_igHe8YH5kP&amp;gclid=Cj0KCQjwuvrBBhDcARIsAKRrkjelT39dppIYbNMYGQDQKVRAcVAnRo2gDZvSJK6NkGomAkksSe1uUHcaAmLSEALw_wcB&amp;gclsrc=aw.ds" xr:uid="{9BDFB2BD-EFF6-4DEE-BBC3-2D01594D0DB0}"/>
-    <hyperlink ref="H22" r:id="rId22" xr:uid="{4FB5C311-0780-4C35-9E62-7B63EE0B1C7F}"/>
-    <hyperlink ref="H19" r:id="rId23" xr:uid="{11D1FB24-874A-4110-8E22-DCAAF354D69C}"/>
-    <hyperlink ref="I2" r:id="rId24" xr:uid="{BB65F326-57F6-0948-9C05-235DDBF32C5D}"/>
-    <hyperlink ref="J2" r:id="rId25" xr:uid="{85148DE2-C5FC-5645-B5BB-41BB837D9E5E}"/>
-    <hyperlink ref="I5" r:id="rId26" xr:uid="{41DE90D8-7589-0C4B-AD96-FF698779CC02}"/>
-    <hyperlink ref="K6" r:id="rId27" xr:uid="{50526146-D5B4-5C42-928A-1A4E698E0A66}"/>
-    <hyperlink ref="I19" r:id="rId28" xr:uid="{FAF305DA-B9D2-2244-A13B-6929AB49025C}"/>
-    <hyperlink ref="I26" r:id="rId29" xr:uid="{B99689F2-D490-2042-A4CC-3BA7CD9172AF}"/>
-    <hyperlink ref="H27" r:id="rId30" xr:uid="{1136733B-68A5-4A0B-995C-2A418A5AC777}"/>
-    <hyperlink ref="I3" r:id="rId31" display="https://www.ebay.com/itm/235081679206?chn=ps&amp;var=536091370095&amp;norover=1&amp;mkevt=1&amp;mkrid=711-117182-37290-0&amp;mkcid=2&amp;mkscid=101&amp;itemid=536091370095_235081679206&amp;targetid=2295557532710&amp;device=c&amp;mktype=pla&amp;googleloc=9198699&amp;poi=&amp;campaignid=21400677539&amp;mkgroupid=173029508628&amp;rlsatarget=pla-2295557532710&amp;abcId=9448483&amp;merchantid=734150552&amp;gad_source=1&amp;gad_campaignid=21400677539&amp;gbraid=0AAAAAD_QDh9KZSet77KcrE8f9gL7cL_CG&amp;gclid=EAIaIQobChMIi8KGzaPsjQMVGEf_AR2yNzdrEAQYAyABEgL6F_D_BwE" xr:uid="{AD11255E-848C-4E6B-B235-2E174E495317}"/>
-    <hyperlink ref="H15" r:id="rId32" xr:uid="{DD127622-0F7B-0F49-8123-68EDBFB9D1FD}"/>
-    <hyperlink ref="I15" r:id="rId33" tooltip="https://www.staples.com/transcend-8gb-microsdhc-memory-card-class-10-ts8gusdhc10/product_IM1LK3226" xr:uid="{CD78FE6E-F962-024D-BECC-56B99B430391}"/>
-    <hyperlink ref="J15" r:id="rId34" tooltip="https://www.cdwg.com/product/transcend-flash-memory-card-8-gb-microsd/3181432?pfm=srh" xr:uid="{F7564EE8-2A81-B244-AEFD-6DA0DF39B5DC}"/>
-    <hyperlink ref="K15" r:id="rId35" tooltip="https://www.cdwg.com/product/kingston-industrial-flash-memory-card-8-gb-microsdhc-uhs-i/6669743?pfm=srh" xr:uid="{6EBC3D1F-2E28-7641-90A9-14D8B6437048}"/>
-    <hyperlink ref="H36" r:id="rId36" xr:uid="{AFFADB06-346C-4E3A-B07A-37D406DF404C}"/>
-    <hyperlink ref="H38" r:id="rId37" xr:uid="{EB0734B3-7C29-4D35-B394-905387802664}"/>
-    <hyperlink ref="H37" r:id="rId38" xr:uid="{26A48533-A061-40FE-A66E-723F0A8526D8}"/>
-    <hyperlink ref="H35" r:id="rId39" xr:uid="{327468E6-6FE8-4274-B476-C9C35280648B}"/>
-    <hyperlink ref="H30" r:id="rId40" display="https://www.digikey.com/en/products/detail/jst-sales-america-inc/B2B-XH-A/1651045?gclsrc=aw.ds&amp;gad_source=1&amp;gad_campaignid=20470400566&amp;gbraid=0AAAAADrbLljaCSzp9mL3BckOGUjmh-pLW&amp;gclid=CjwKCAiAoNbIBhB5EiwAZFbYGEhTlbpU8AtASh9T03rT2O-as-UbMvwFZowiONL1Xf91TSJaIz9zzBoCD-IQAvD_BwE" xr:uid="{A1578E18-966D-4A0B-89BB-AAA405790B24}"/>
-    <hyperlink ref="H7" r:id="rId41" xr:uid="{809BB693-6445-43CC-B4C1-47C121254BDE}"/>
-    <hyperlink ref="I7" r:id="rId42" xr:uid="{8E7D6AC4-E51D-48DC-AC39-840AA30DB295}"/>
-    <hyperlink ref="H21" r:id="rId43" xr:uid="{F2FBC813-F21B-4CA5-94D5-A1D3C7097891}"/>
-    <hyperlink ref="H13" r:id="rId44" xr:uid="{0C1E97B9-B29C-4292-84AE-9AEFCCB0C868}"/>
-    <hyperlink ref="H18" r:id="rId45" xr:uid="{51407470-A2C9-4C4E-89CA-FC24B70AF5A7}"/>
-    <hyperlink ref="I4" r:id="rId46" xr:uid="{1A2534D8-294F-4B39-89B1-8168C50C4225}"/>
-    <hyperlink ref="L6" r:id="rId47" xr:uid="{3B26DD18-290E-4BFE-BB80-46E0A92D8884}"/>
-    <hyperlink ref="J6" r:id="rId48" display="https://www.ebay.com/itm/223602242983?chn=ps&amp;norover=1&amp;mkevt=1&amp;mkrid=711-117182-37290-0&amp;mkcid=2&amp;mkscid=101&amp;itemid=223602242983&amp;targetid=2295557532710&amp;device=c&amp;mktype=pla&amp;googleloc=9198699&amp;poi=&amp;campaignid=21400677539&amp;mkgroupid=173029508628&amp;rlsatarget=pla-2295557532710&amp;abcId=9448483&amp;merchantid=108461346&amp;gad_source=4&amp;gad_campaignid=21400677539&amp;gbraid=0AAAAAD_QDh9zBpIZmq8atlokvhUYT34hx&amp;gclid=EAIaIQobChMIyYbmlabsjQMVBjUIBR1KhTUNEAQYECABEgIh5fD_BwE" xr:uid="{8537022B-3B72-40E4-A752-C847F511BEE6}"/>
-    <hyperlink ref="I10" r:id="rId49" xr:uid="{637C6DC6-6221-421C-AA28-8557881CF9FD}"/>
-    <hyperlink ref="H6" r:id="rId50" display="https://www.ebay.com/itm/327147846952?_skw=BME280+5+V&amp;itmmeta=01KZVT1RTW26G1WWC3Y7NSNY2T&amp;hash=item4c2b87fd28:g:P1MAAeSwcWdp~jCK&amp;itmprp=enc%3AAQALAAAA8GfYFPkwiKCW4ZNSs2u11xBLJ1nUqR2xZVn5ICoE5NiiwYxCuP3oV0tHbDyiTrJD6bhCyVqNwlfr2mQRgt69x13oWtdQi3TcBKAuALu5BNc4kizG71QWWkAnkaRzxc93ZvydEM%2FyrxyG14dVHixNOtgOl7X2xvEDeCMFXXRaGsjHeDjGqmK2jMUC9ka7BsCHxyMshnuNFyognz3gtR%2BWK1dTMlzpuPDICn17tBE%2FFpZy32gKf86YoyfEdoW%2F4ljDIFbON%2Fpdh3orFKZz8nXCSJ2jXq6V4mpyIF%2FyoDRezAxZEhVOZPmSQyEnnuyLp49zGQ%3D%3D%7Ctkp%3ABFBM2I2H-v5n" xr:uid="{B10E6281-8922-4D98-84C4-5D848CF9F0D8}"/>
+    <hyperlink ref="H4" r:id="rId1" display="https://www.amazon.com/Makerfire-Arduino-NRF24L01-Wireless-Transceiver/dp/B00O9O868G/ref=asc_df_B00O9O868G?mcid=dab308f0de3430dfa5c9f8399ca22b35&amp;hvocijid=9184541888213339040-B00O9O868G-&amp;hvexpln=73&amp;tag=hyprod-20&amp;linkCode=df0&amp;hvadid=721245378154&amp;hvpos=&amp;hvnetw=g&amp;hvrand=9184541888213339040&amp;hvpone=&amp;hvptwo=&amp;hvqmt=&amp;hvdev=c&amp;hvdvcmdl=&amp;hvlocint=&amp;hvlocphy=9198699&amp;hvtargid=pla-2281435177578&amp;psc=1" xr:uid="{89AEDB65-21E6-41D2-A940-81A81142AD5C}"/>
+    <hyperlink ref="H5" r:id="rId2" xr:uid="{E70F36E4-82C7-490A-965C-FBA0B568208C}"/>
+    <hyperlink ref="I6" r:id="rId3" display="https://www.amazon.com/Onyehn-Temperature-Humidity-Barometric-Pressure/dp/B07KR24P6P/ref=asc_df_B07KR24P6P?mcid=2faf80a473c33e3bb7b53dc75a65a9ac&amp;hvocijid=2199110702432476394-B07KR24P6P-&amp;hvexpln=73&amp;tag=hyprod-20&amp;linkCode=df0&amp;hvadid=721245378154&amp;hvpos=&amp;hvnetw=g&amp;hvrand=2199110702432476394&amp;hvpone=&amp;hvptwo=&amp;hvqmt=&amp;hvdev=c&amp;hvdvcmdl=&amp;hvlocint=&amp;hvlocphy=9198699&amp;hvtargid=pla-2281435177578&amp;psc=1" xr:uid="{04CEC65C-3665-4D25-B259-AF9E667F3BA6}"/>
+    <hyperlink ref="H8" r:id="rId4" xr:uid="{23E423E1-1EBE-4115-AE06-49032C41D232}"/>
+    <hyperlink ref="H9" r:id="rId5" display="https://www.sparkfun.com/ultrasonic-distance-sensor-hc-sr04.html" xr:uid="{F999829F-3DFC-4DBA-B819-1D673798FA55}"/>
+    <hyperlink ref="H10" r:id="rId6" display="https://zeeebattery.com/products/zeee-7-4v-60c-1500mah-2s-lipo-battery-deans-plug?variant=43953770299699&amp;country=US&amp;currency=USD&amp;utm_medium=product_sync&amp;utm_source=google&amp;utm_content=sag_organic&amp;utm_campaign=sag_organic&amp;gad_source=1&amp;gclid=CjwKCAjw7pO_BhAlEiwA4pMQvJInDAYww1F-RyBS_FKHJZs2q-GgKMjZj0IEfHsjSMYCjfxmAI9laxoCeRQQAvD_BwE" xr:uid="{BB8CB9D1-9310-4C54-A510-64D6DA058543}"/>
+    <hyperlink ref="H11" r:id="rId7" display="https://www.digikey.com/en/products/detail/jauch-quartz/CR1025/16399048" xr:uid="{17A29435-522E-4BB5-8364-3BC77FBEB1C4}"/>
+    <hyperlink ref="H12" r:id="rId8" display="https://www.digikey.com/en/products/detail/mpd-memory-protection-devices/bk-870/3829737" xr:uid="{27F9BEB5-8046-41B8-A401-6B801AA65292}"/>
+    <hyperlink ref="H17" r:id="rId9" display="https://www.digikey.com/en/products/detail/american-opto-plus-led/L314ED/13677700?s=N4IgTCBcDaIDIGYCMAWAogERAXQL5A" xr:uid="{EB1FB783-CD78-4F2E-ADAE-2EFC2E0C050D}"/>
+    <hyperlink ref="H20" r:id="rId10" xr:uid="{1CE23A94-3355-4CE3-BD99-944097BF2C76}"/>
+    <hyperlink ref="H25" r:id="rId11" display="https://www.digikey.com/en/products/detail/kemet/c1206s104k5racauto/10232834" xr:uid="{CDDFAE49-11BE-4283-9E44-D17951ACE335}"/>
+    <hyperlink ref="H26" r:id="rId12" display="https://www.digikey.com/en/products/detail/microchip-technology/mic5239-5-0ys-tr/2346595" xr:uid="{0FF0C8FA-B521-42B4-9637-4551CDF56AE0}"/>
+    <hyperlink ref="H28" r:id="rId13" display="https://www.digikey.com/en/products/detail/samtec-inc/ssa-104-w-t/1105908" xr:uid="{5CEFEAD0-E765-4C5C-8B17-4D481AAEE74F}"/>
+    <hyperlink ref="H14" r:id="rId14" xr:uid="{98CBDFFF-5BC0-4691-985C-193C55CD2A4F}"/>
+    <hyperlink ref="H16" r:id="rId15" xr:uid="{F40F3420-CF30-4700-92F3-040B50F37E84}"/>
+    <hyperlink ref="H23" r:id="rId16" xr:uid="{CF84383E-32DC-4F7A-8B1F-D5487EDC174E}"/>
+    <hyperlink ref="H24" r:id="rId17" xr:uid="{9AFC6348-0E57-4A67-A197-41D4FD45794D}"/>
+    <hyperlink ref="H3" r:id="rId18" xr:uid="{132AA37F-9E12-44EF-9546-36BDCE2F9F6B}"/>
+    <hyperlink ref="H32" r:id="rId19" xr:uid="{BECD5DE6-8852-4EA8-869E-7E18A46D5C74}"/>
+    <hyperlink ref="H31" r:id="rId20" display="https://www.digikey.com/en/products/detail/jst-sales-america-inc/B3B-XH-A/1651046?gad_source=1&amp;gad_campaignid=20470400566&amp;gbraid=0AAAAADrbLlgCz6Py2S0va5_igHe8YH5kP&amp;gclid=Cj0KCQjwuvrBBhDcARIsAKRrkjelT39dppIYbNMYGQDQKVRAcVAnRo2gDZvSJK6NkGomAkksSe1uUHcaAmLSEALw_wcB&amp;gclsrc=aw.ds" xr:uid="{9BDFB2BD-EFF6-4DEE-BBC3-2D01594D0DB0}"/>
+    <hyperlink ref="H22" r:id="rId21" xr:uid="{4FB5C311-0780-4C35-9E62-7B63EE0B1C7F}"/>
+    <hyperlink ref="H19" r:id="rId22" xr:uid="{11D1FB24-874A-4110-8E22-DCAAF354D69C}"/>
+    <hyperlink ref="I5" r:id="rId23" xr:uid="{41DE90D8-7589-0C4B-AD96-FF698779CC02}"/>
+    <hyperlink ref="K6" r:id="rId24" xr:uid="{50526146-D5B4-5C42-928A-1A4E698E0A66}"/>
+    <hyperlink ref="I19" r:id="rId25" xr:uid="{FAF305DA-B9D2-2244-A13B-6929AB49025C}"/>
+    <hyperlink ref="I26" r:id="rId26" xr:uid="{B99689F2-D490-2042-A4CC-3BA7CD9172AF}"/>
+    <hyperlink ref="H27" r:id="rId27" xr:uid="{1136733B-68A5-4A0B-995C-2A418A5AC777}"/>
+    <hyperlink ref="I3" r:id="rId28" display="https://www.ebay.com/itm/235081679206?chn=ps&amp;var=536091370095&amp;norover=1&amp;mkevt=1&amp;mkrid=711-117182-37290-0&amp;mkcid=2&amp;mkscid=101&amp;itemid=536091370095_235081679206&amp;targetid=2295557532710&amp;device=c&amp;mktype=pla&amp;googleloc=9198699&amp;poi=&amp;campaignid=21400677539&amp;mkgroupid=173029508628&amp;rlsatarget=pla-2295557532710&amp;abcId=9448483&amp;merchantid=734150552&amp;gad_source=1&amp;gad_campaignid=21400677539&amp;gbraid=0AAAAAD_QDh9KZSet77KcrE8f9gL7cL_CG&amp;gclid=EAIaIQobChMIi8KGzaPsjQMVGEf_AR2yNzdrEAQYAyABEgL6F_D_BwE" xr:uid="{AD11255E-848C-4E6B-B235-2E174E495317}"/>
+    <hyperlink ref="H15" r:id="rId29" xr:uid="{DD127622-0F7B-0F49-8123-68EDBFB9D1FD}"/>
+    <hyperlink ref="I15" r:id="rId30" tooltip="https://www.staples.com/transcend-8gb-microsdhc-memory-card-class-10-ts8gusdhc10/product_IM1LK3226" xr:uid="{CD78FE6E-F962-024D-BECC-56B99B430391}"/>
+    <hyperlink ref="J15" r:id="rId31" tooltip="https://www.cdwg.com/product/transcend-flash-memory-card-8-gb-microsd/3181432?pfm=srh" xr:uid="{F7564EE8-2A81-B244-AEFD-6DA0DF39B5DC}"/>
+    <hyperlink ref="K15" r:id="rId32" tooltip="https://www.cdwg.com/product/kingston-industrial-flash-memory-card-8-gb-microsdhc-uhs-i/6669743?pfm=srh" xr:uid="{6EBC3D1F-2E28-7641-90A9-14D8B6437048}"/>
+    <hyperlink ref="H36" r:id="rId33" xr:uid="{AFFADB06-346C-4E3A-B07A-37D406DF404C}"/>
+    <hyperlink ref="H38" r:id="rId34" xr:uid="{EB0734B3-7C29-4D35-B394-905387802664}"/>
+    <hyperlink ref="H37" r:id="rId35" xr:uid="{26A48533-A061-40FE-A66E-723F0A8526D8}"/>
+    <hyperlink ref="H35" r:id="rId36" xr:uid="{327468E6-6FE8-4274-B476-C9C35280648B}"/>
+    <hyperlink ref="H30" r:id="rId37" display="https://www.digikey.com/en/products/detail/jst-sales-america-inc/B2B-XH-A/1651045?gclsrc=aw.ds&amp;gad_source=1&amp;gad_campaignid=20470400566&amp;gbraid=0AAAAADrbLljaCSzp9mL3BckOGUjmh-pLW&amp;gclid=CjwKCAiAoNbIBhB5EiwAZFbYGEhTlbpU8AtASh9T03rT2O-as-UbMvwFZowiONL1Xf91TSJaIz9zzBoCD-IQAvD_BwE" xr:uid="{A1578E18-966D-4A0B-89BB-AAA405790B24}"/>
+    <hyperlink ref="H7" r:id="rId38" xr:uid="{809BB693-6445-43CC-B4C1-47C121254BDE}"/>
+    <hyperlink ref="I7" r:id="rId39" xr:uid="{8E7D6AC4-E51D-48DC-AC39-840AA30DB295}"/>
+    <hyperlink ref="H21" r:id="rId40" xr:uid="{F2FBC813-F21B-4CA5-94D5-A1D3C7097891}"/>
+    <hyperlink ref="H13" r:id="rId41" xr:uid="{0C1E97B9-B29C-4292-84AE-9AEFCCB0C868}"/>
+    <hyperlink ref="H18" r:id="rId42" xr:uid="{51407470-A2C9-4C4E-89CA-FC24B70AF5A7}"/>
+    <hyperlink ref="I4" r:id="rId43" xr:uid="{1A2534D8-294F-4B39-89B1-8168C50C4225}"/>
+    <hyperlink ref="L6" r:id="rId44" xr:uid="{3B26DD18-290E-4BFE-BB80-46E0A92D8884}"/>
+    <hyperlink ref="J6" r:id="rId45" display="https://www.ebay.com/itm/223602242983?chn=ps&amp;norover=1&amp;mkevt=1&amp;mkrid=711-117182-37290-0&amp;mkcid=2&amp;mkscid=101&amp;itemid=223602242983&amp;targetid=2295557532710&amp;device=c&amp;mktype=pla&amp;googleloc=9198699&amp;poi=&amp;campaignid=21400677539&amp;mkgroupid=173029508628&amp;rlsatarget=pla-2295557532710&amp;abcId=9448483&amp;merchantid=108461346&amp;gad_source=4&amp;gad_campaignid=21400677539&amp;gbraid=0AAAAAD_QDh9zBpIZmq8atlokvhUYT34hx&amp;gclid=EAIaIQobChMIyYbmlabsjQMVBjUIBR1KhTUNEAQYECABEgIh5fD_BwE" xr:uid="{8537022B-3B72-40E4-A752-C847F511BEE6}"/>
+    <hyperlink ref="I10" r:id="rId46" xr:uid="{637C6DC6-6221-421C-AA28-8557881CF9FD}"/>
+    <hyperlink ref="H6" r:id="rId47" display="https://www.ebay.com/itm/327147846952?_skw=BME280+5+V&amp;itmmeta=01KZVT1RTW26G1WWC3Y7NSNY2T&amp;hash=item4c2b87fd28:g:P1MAAeSwcWdp~jCK&amp;itmprp=enc%3AAQALAAAA8GfYFPkwiKCW4ZNSs2u11xBLJ1nUqR2xZVn5ICoE5NiiwYxCuP3oV0tHbDyiTrJD6bhCyVqNwlfr2mQRgt69x13oWtdQi3TcBKAuALu5BNc4kizG71QWWkAnkaRzxc93ZvydEM%2FyrxyG14dVHixNOtgOl7X2xvEDeCMFXXRaGsjHeDjGqmK2jMUC9ka7BsCHxyMshnuNFyognz3gtR%2BWK1dTMlzpuPDICn17tBE%2FFpZy32gKf86YoyfEdoW%2F4ljDIFbON%2Fpdh3orFKZz8nXCSJ2jXq6V4mpyIF%2FyoDRezAxZEhVOZPmSQyEnnuyLp49zGQ%3D%3D%7Ctkp%3ABFBM2I2H-v5n" xr:uid="{B10E6281-8922-4D98-84C4-5D848CF9F0D8}"/>
+    <hyperlink ref="H2" r:id="rId48" xr:uid="{08416717-5082-4BB2-87F2-3F9086D6C942}"/>
+    <hyperlink ref="I2" r:id="rId49" display="https://www.sparkfun.com/arduino-nano-every.html?utm_source=google&amp;utm_medium=cpc&amp;utm_campaign=Generic+%7C+PMax&amp;utm_content=Full+Catalog&amp;gad_source=1&amp;gad_campaignid=17479024039&amp;gbraid=0AAAAADsj4ET0NZro45iUWdM-Ba6AQ0YWk&amp;gclid=CjwKCAjw_KjVBhAHEiwAnC0N9MHYi96OUVs8ZOLr9cRyVdCITPEBJ4SesPMJTw66NdfeWCyuEPozBxoCvzYQAvD_BwE" xr:uid="{ED6E6F72-D42D-4092-930B-8B8FBCA70E05}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId51"/>
+  <pageSetup orientation="portrait" r:id="rId50"/>
 </worksheet>
 </file>
</xml_diff>